<commit_message>
Items, vendors, stores CRUD and Testing all completed
</commit_message>
<xml_diff>
--- a/WorkBot/main/data/orders/Hill & Markes/Hill & Markes_Bakery_20260601.xlsx
+++ b/WorkBot/main/data/orders/Hill & Markes/Hill & Markes_Bakery_20260601.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,6 +542,363 @@
         <v>100.28</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DUO71006</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bag - Paper (6#)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="E9" t="n">
+        <v>12.78</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DUO71010</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bag - Paper (10#)</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="E10" t="n">
+        <v>12.78</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SMTSM2PIKN</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Napkin - Dispenser</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>25.16</v>
+      </c>
+      <c r="E11" t="n">
+        <v>25.16</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>INLSLP17XD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Container - Plastic Eclair</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>87.93000000000001</v>
+      </c>
+      <c r="E12" t="n">
+        <v>87.93000000000001</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CC-802</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cup Carrier - Fiber (2-Cup)</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>14.82</v>
+      </c>
+      <c r="E13" t="n">
+        <v>14.82</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TS8</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Tamper Evident - 8oz</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>41.36</v>
+      </c>
+      <c r="E14" t="n">
+        <v>206.8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>KLP704534</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Trash Bag (33x40)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>24.27</v>
+      </c>
+      <c r="E15" t="n">
+        <v>24.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SPT460200</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Hand Soap - Foaming</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>43.86</v>
+      </c>
+      <c r="E16" t="n">
+        <v>43.86</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NPP406020</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Spoon Soup - White MW</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="n">
+        <v>10.2</v>
+      </c>
+      <c r="E17" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>508</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bag - Wax (Sandwich)</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>113.57</v>
+      </c>
+      <c r="E18" t="n">
+        <v>113.57</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>FLOW15</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wrap - Paper (15" x 10.75")</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="E19" t="n">
+        <v>143.2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>FWW6</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Wrap - Paper (6" x 10.75")</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>93.40000000000001</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>INPSDR0200ITHACABAKERY</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cup - Hot (20oz)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>83.13</v>
+      </c>
+      <c r="E21" t="n">
+        <v>83.13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>INPSDR0160ITHACABAKERY</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Cup - Hot (16oz)</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>70.09</v>
+      </c>
+      <c r="E22" t="n">
+        <v>70.09</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>INPSDR0120ITHACABAKERY</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Cup - Hot (12oz)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>62.78</v>
+      </c>
+      <c r="E23" t="n">
+        <v>62.78</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AVLJNA26W</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Straws - Wrapped</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>53.54</v>
+      </c>
+      <c r="E24" t="n">
+        <v>107.08</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>INPSMR0080SH</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cup - Hot (8oz)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>54.5</v>
+      </c>
+      <c r="E25" t="n">
+        <v>54.5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>